<commit_message>
Add hardware-aware generation and source handling
Add hardware.source with hardware-aware power allocation and validation
Add structured hardware compatibility diagnostics and candidate rejection reporting
Standardize biased-pulse stress on pulse_width with a 10 ms REALIS default
Support literal, referenced, and templated DUT names from project metadata
Resolve relative source paths from the generation file location
Add Excel-backed source and hardware configuration examples
</commit_message>
<xml_diff>
--- a/examples/sources/spreadsheet_pin_source/data/customer-device.xlsx
+++ b/examples/sources/spreadsheet_pin_source/data/customer-device.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="1" r:id="R19acc703183d4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pins" sheetId="1" r:id="Rdd774a8e929a4c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project" sheetId="2" r:id="R7fe99d914b85407d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27,12 +28,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -47,7 +53,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -55,6 +61,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -369,4 +378,40 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.880000114440918" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>project_name</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str">
+        <x:v>product_basic_type</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="str">
+        <x:v>sales_code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Spreadsheet Source Demo</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>CUSTOMER-IC-42</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>DEMO-42</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>